<commit_message>
fix 950 custom ops compile  func
</commit_message>
<xml_diff>
--- a/csrc/attention/compressor/tests/pytest/excel/example.xlsx
+++ b/csrc/attention/compressor/tests/pytest/excel/example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20398"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20416"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\cann\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\c00936096\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5969243-5160-4753-A22A-F1FDBF75D033}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FE0C103-ED8F-403B-AD70-1E2B1264D461}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -170,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -178,9 +178,11 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -499,15 +501,15 @@
   <dimension ref="A1:Y3"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="13.625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="11" width="13.625" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.625" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.625" style="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="13.625" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.625" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.625" style="5" bestFit="1" customWidth="1"/>
-    <col min="19" max="24" width="13.625" style="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.25" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="11" width="13.625" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.625" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.625" style="9" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="13.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.625" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.625" style="7" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="13.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.25" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -547,7 +549,7 @@
       <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
@@ -591,40 +593,40 @@
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="4">
         <v>1</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="4">
         <v>4096</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="4">
         <v>8192</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>512</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="4">
         <v>128</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="4">
         <v>64</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="4">
         <v>4</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="4">
         <v>2</v>
       </c>
-      <c r="J2" s="3">
+      <c r="J2" s="4">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="4">
         <v>0</v>
       </c>
       <c r="L2" s="2">
         <v>2</v>
       </c>
-      <c r="M2" s="2">
+      <c r="M2" s="5">
         <v>1</v>
       </c>
       <c r="N2" s="1" t="s">
@@ -635,7 +637,7 @@
       </c>
       <c r="P2" s="1"/>
       <c r="Q2" s="2"/>
-      <c r="R2" s="3"/>
+      <c r="R2" s="4"/>
       <c r="S2" s="1" t="s">
         <v>28</v>
       </c>
@@ -662,40 +664,40 @@
       <c r="A3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="4">
         <v>1</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="4">
         <v>4096</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="4">
         <v>8192</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="4">
         <v>128</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="4">
         <v>128</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="4">
         <v>64</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="4">
         <v>4</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="4">
         <v>2</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="4">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="4">
         <v>0</v>
       </c>
       <c r="L3" s="2">
         <v>2</v>
       </c>
-      <c r="M3" s="2">
+      <c r="M3" s="5">
         <v>1</v>
       </c>
       <c r="N3" s="1" t="s">
@@ -710,7 +712,7 @@
       <c r="Q3" s="2">
         <v>2</v>
       </c>
-      <c r="R3" s="3">
+      <c r="R3" s="4">
         <v>8192</v>
       </c>
       <c r="S3" s="1" t="s">

</xml_diff>

<commit_message>
Add A5 FP8 quantization support for DSA attention
</commit_message>
<xml_diff>
--- a/csrc/attention/compressor/tests/pytest/excel/example.xlsx
+++ b/csrc/attention/compressor/tests/pytest/excel/example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20398"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20416"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\cann\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\c00936096\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5969243-5160-4753-A22A-F1FDBF75D033}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FE0C103-ED8F-403B-AD70-1E2B1264D461}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -170,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -178,9 +178,11 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -499,15 +501,15 @@
   <dimension ref="A1:Y3"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="13.625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="11" width="13.625" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.625" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.625" style="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="13.625" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.625" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.625" style="5" bestFit="1" customWidth="1"/>
-    <col min="19" max="24" width="13.625" style="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.25" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="11" width="13.625" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.625" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.625" style="9" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="13.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.625" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.625" style="7" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="13.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.25" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -547,7 +549,7 @@
       <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
@@ -591,40 +593,40 @@
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="4">
         <v>1</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="4">
         <v>4096</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="4">
         <v>8192</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>512</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="4">
         <v>128</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="4">
         <v>64</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="4">
         <v>4</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="4">
         <v>2</v>
       </c>
-      <c r="J2" s="3">
+      <c r="J2" s="4">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="4">
         <v>0</v>
       </c>
       <c r="L2" s="2">
         <v>2</v>
       </c>
-      <c r="M2" s="2">
+      <c r="M2" s="5">
         <v>1</v>
       </c>
       <c r="N2" s="1" t="s">
@@ -635,7 +637,7 @@
       </c>
       <c r="P2" s="1"/>
       <c r="Q2" s="2"/>
-      <c r="R2" s="3"/>
+      <c r="R2" s="4"/>
       <c r="S2" s="1" t="s">
         <v>28</v>
       </c>
@@ -662,40 +664,40 @@
       <c r="A3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="4">
         <v>1</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="4">
         <v>4096</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="4">
         <v>8192</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="4">
         <v>128</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="4">
         <v>128</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="4">
         <v>64</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="4">
         <v>4</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="4">
         <v>2</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="4">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="4">
         <v>0</v>
       </c>
       <c r="L3" s="2">
         <v>2</v>
       </c>
-      <c r="M3" s="2">
+      <c r="M3" s="5">
         <v>1</v>
       </c>
       <c r="N3" s="1" t="s">
@@ -710,7 +712,7 @@
       <c r="Q3" s="2">
         <v>2</v>
       </c>
-      <c r="R3" s="3">
+      <c r="R3" s="4">
         <v>8192</v>
       </c>
       <c r="S3" s="1" t="s">

</xml_diff>